<commit_message>
Record results of the refreshed HBAN code test
- tools/update_catalog.py: mark codes that returned numbers in a refreshed workbook as
  VERIFIED in the catalog (positive evidence only; appends missing codes)
- catalog: 28 codes newly verified (FB fallbacks, FFI NPL/NIM/leverage, FF tier 1 /
  capital ratios, FF_DIV_CF, FF_BK_COM_EQ_TIER1_TOT added); warnings for leverage 99.95,
  cost-of-funds duplicates, NETCHARGE_LOANNET #NUM!, COM_EQUITY_TIER1 time series, loan outliers
- guide: cross-family @ chains are proven; chain takes the first number even if wrong;
  FE horizon notes; CAMELS table ticks updated
- sample workbook: statuses rebuilt from the updated catalog

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TZGHEwBk7ZqkzJs7eP5z1i
</commit_message>
<xml_diff>
--- a/samples/HBAN_FDS_Code_Test_SAMPLE.xlsx
+++ b/samples/HBAN_FDS_Code_Test_SAMPLE.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="167" formatCode="#,##0.00&quot;%&quot;_);(#,##0.00&quot;%&quot;)"/>
     <numFmt numFmtId="168" formatCode="$#,##0.00#_);($#,##0.00#)"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,17 +80,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="FFB26A00"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <color rgb="FF595959"/>
       <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="FFB00B1C"/>
+      <color rgb="FFB26A00"/>
       <sz val="8"/>
     </font>
     <font>
@@ -140,12 +135,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -168,15 +163,14 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="39" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="37" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -552,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -651,7 +645,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">                       3 global banks (HSBA-GB, SAN-ES, NAB-AU). Tests whether cross-family chains work.</t>
+          <t xml:space="preserve">                       3 global banks (HSBA-GB, SAN-ES, NAB-AU). Shows which family works per bank.</t>
         </is>
       </c>
     </row>
@@ -703,43 +697,50 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Unproven chain  cross-family @ fallback (FFI@FF@FB) - check it fills in where a single family works.</t>
+          <t>Chain           cross-family @ fallback (FFI@FF@FB) - proven in the Oct 2026 refresh; takes the first</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">                family that returns a number, even a wrong one (check outliers).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
           <t>Cell math       calculated in Excel from the rows above.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Units</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>$ in millions; per-share in $; % as whole numbers (10.5 = 10.5%). NCO ratio and deposit cost are</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>quarterly rates x4; FF_EFF_RATIO is a fraction x100. FB_ codes cover US banks only.</t>
+          <t>$ in millions; per-share in $; % as whole numbers (10.5 = 10.5%). NCO ratio and deposit cost are</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>quarterly rates x4; FF_EFF_RATIO is a fraction x100. FB_ codes cover US banks only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Outside Excel+FactSet every formula shows #NAME? - that is expected.</t>
         </is>
@@ -1277,9 +1278,9 @@
           <t>FF_DIV_CF(QTR,{p})</t>
         </is>
       </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E19" s="17">
@@ -1358,23 +1359,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E21" s="20">
+      <c r="E21" s="19">
         <f>_xlfn.IFNA(FDS(E$6,"FF_DPS(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="F21" s="20">
+      <c r="F21" s="19">
         <f>_xlfn.IFNA(FDS(F$6,"FF_DPS(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="G21" s="20">
+      <c r="G21" s="19">
         <f>_xlfn.IFNA(FDS(G$6,"FF_DPS(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="H21" s="20">
+      <c r="H21" s="19">
         <f>_xlfn.IFNA(FDS(H$6,"FF_DPS(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="I21" s="20">
+      <c r="I21" s="19">
         <f>_xlfn.IFNA(FDS(I$6,"FF_DPS(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
@@ -1396,23 +1397,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E22" s="21">
+      <c r="E22" s="20">
         <f>_xlfn.IFNA(FDS(E$6,"FF_COM_SHS_OUT(QTR_R,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="F22" s="21">
+      <c r="F22" s="20">
         <f>_xlfn.IFNA(FDS(F$6,"FF_COM_SHS_OUT(QTR_R,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="G22" s="21">
+      <c r="G22" s="20">
         <f>_xlfn.IFNA(FDS(G$6,"FF_COM_SHS_OUT(QTR_R,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="H22" s="21">
+      <c r="H22" s="20">
         <f>_xlfn.IFNA(FDS(H$6,"FF_COM_SHS_OUT(QTR_R,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="I22" s="21">
+      <c r="I22" s="20">
         <f>_xlfn.IFNA(FDS(I$6,"FF_COM_SHS_OUT(QTR_R,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
@@ -1639,23 +1640,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E29" s="20">
+      <c r="E29" s="19">
         <f>_xlfn.IFNA(FDS(E$6,"FF_EPS(QTR_R,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="F29" s="20">
+      <c r="F29" s="19">
         <f>_xlfn.IFNA(FDS(F$6,"FF_EPS(QTR_R,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="G29" s="20">
+      <c r="G29" s="19">
         <f>_xlfn.IFNA(FDS(G$6,"FF_EPS(QTR_R,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="H29" s="20">
+      <c r="H29" s="19">
         <f>_xlfn.IFNA(FDS(H$6,"FF_EPS(QTR_R,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="I29" s="20">
+      <c r="I29" s="19">
         <f>_xlfn.IFNA(FDS(I$6,"FF_EPS(QTR_R,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
@@ -2953,23 +2954,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E66" s="20">
+      <c r="E66" s="19">
         <f>_xlfn.IFNA(FDS(E$6,"FF_BPS_TANG(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="F66" s="20">
+      <c r="F66" s="19">
         <f>_xlfn.IFNA(FDS(F$6,"FF_BPS_TANG(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="G66" s="20">
+      <c r="G66" s="19">
         <f>_xlfn.IFNA(FDS(G$6,"FF_BPS_TANG(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="H66" s="20">
+      <c r="H66" s="19">
         <f>_xlfn.IFNA(FDS(H$6,"FF_BPS_TANG(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="I66" s="20">
+      <c r="I66" s="19">
         <f>_xlfn.IFNA(FDS(I$6,"FF_BPS_TANG(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
@@ -3226,23 +3227,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E75" s="22">
+      <c r="E75" s="21">
         <f>_xlfn.IFNA(FDS(E$6,"FB_DOM_OFFCE_NUM(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="F75" s="22">
+      <c r="F75" s="21">
         <f>_xlfn.IFNA(FDS(F$6,"FB_DOM_OFFCE_NUM(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="G75" s="22">
+      <c r="G75" s="21">
         <f>_xlfn.IFNA(FDS(G$6,"FB_DOM_OFFCE_NUM(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="H75" s="22">
+      <c r="H75" s="21">
         <f>_xlfn.IFNA(FDS(H$6,"FB_DOM_OFFCE_NUM(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="I75" s="22">
+      <c r="I75" s="21">
         <f>_xlfn.IFNA(FDS(I$6,"FB_DOM_OFFCE_NUM(QTR,"&amp;$C$3&amp;")"),"-")</f>
         <v/>
       </c>
@@ -3279,23 +3280,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E77" s="20">
+      <c r="E77" s="19">
         <f>_xlfn.IFNA(FDS(E$6,"FE_ESTIMATE(EPS_NONGAAP,MEAN,QTR,"&amp;$C$3&amp;",0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="F77" s="20">
+      <c r="F77" s="19">
         <f>_xlfn.IFNA(FDS(F$6,"FE_ESTIMATE(EPS_NONGAAP,MEAN,QTR,"&amp;$C$3&amp;",0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="G77" s="20">
+      <c r="G77" s="19">
         <f>_xlfn.IFNA(FDS(G$6,"FE_ESTIMATE(EPS_NONGAAP,MEAN,QTR,"&amp;$C$3&amp;",0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="H77" s="20">
+      <c r="H77" s="19">
         <f>_xlfn.IFNA(FDS(H$6,"FE_ESTIMATE(EPS_NONGAAP,MEAN,QTR,"&amp;$C$3&amp;",0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="I77" s="20">
+      <c r="I77" s="19">
         <f>_xlfn.IFNA(FDS(I$6,"FE_ESTIMATE(EPS_NONGAAP,MEAN,QTR,"&amp;$C$3&amp;",0,,,'')"),"-")</f>
         <v/>
       </c>
@@ -3543,7 +3544,7 @@
           <t>Ticker</t>
         </is>
       </c>
-      <c r="C3" s="23" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>HBAN</t>
         </is>
@@ -3612,49 +3613,49 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>Prior quarter (TSR start)</t>
         </is>
       </c>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="24" t="n"/>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="C6" s="23" t="n"/>
+      <c r="D6" s="23" t="n"/>
+      <c r="E6" s="23" t="inlineStr">
         <is>
           <t>2024/2F</t>
         </is>
       </c>
-      <c r="F6" s="24" t="inlineStr">
+      <c r="F6" s="23" t="inlineStr">
         <is>
           <t>2024/3F</t>
         </is>
       </c>
-      <c r="G6" s="24" t="inlineStr">
+      <c r="G6" s="23" t="inlineStr">
         <is>
           <t>2024/4F</t>
         </is>
       </c>
-      <c r="H6" s="24" t="inlineStr">
+      <c r="H6" s="23" t="inlineStr">
         <is>
           <t>2025/1F</t>
         </is>
       </c>
-      <c r="I6" s="24" t="inlineStr">
+      <c r="I6" s="23" t="inlineStr">
         <is>
           <t>2025/2F</t>
         </is>
       </c>
-      <c r="J6" s="24" t="inlineStr">
+      <c r="J6" s="23" t="inlineStr">
         <is>
           <t>2025/3F</t>
         </is>
       </c>
-      <c r="K6" s="24" t="inlineStr">
+      <c r="K6" s="23" t="inlineStr">
         <is>
           <t>2025/4F</t>
         </is>
       </c>
-      <c r="L6" s="24" t="inlineStr">
+      <c r="L6" s="23" t="inlineStr">
         <is>
           <t>2026/1F</t>
         </is>
@@ -4158,9 +4159,9 @@
           <t>FF_DIV_CF(QTR,{p})</t>
         </is>
       </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E19" s="17">
@@ -4263,35 +4264,35 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E21" s="20">
+      <c r="E21" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_DPS(QTR,"&amp;E$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="F21" s="20">
+      <c r="F21" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_DPS(QTR,"&amp;F$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="G21" s="20">
+      <c r="G21" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_DPS(QTR,"&amp;G$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="H21" s="20">
+      <c r="H21" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_DPS(QTR,"&amp;H$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="I21" s="20">
+      <c r="I21" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_DPS(QTR,"&amp;I$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="J21" s="20">
+      <c r="J21" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_DPS(QTR,"&amp;J$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="K21" s="20">
+      <c r="K21" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_DPS(QTR,"&amp;K$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="L21" s="20">
+      <c r="L21" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_DPS(QTR,"&amp;L$5&amp;")"),"-")</f>
         <v/>
       </c>
@@ -4313,35 +4314,35 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E22" s="21">
+      <c r="E22" s="20">
         <f>_xlfn.IFNA(FDS($C$3,"FF_COM_SHS_OUT(QTR_R,"&amp;E$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="F22" s="21">
+      <c r="F22" s="20">
         <f>_xlfn.IFNA(FDS($C$3,"FF_COM_SHS_OUT(QTR_R,"&amp;F$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="G22" s="21">
+      <c r="G22" s="20">
         <f>_xlfn.IFNA(FDS($C$3,"FF_COM_SHS_OUT(QTR_R,"&amp;G$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="H22" s="21">
+      <c r="H22" s="20">
         <f>_xlfn.IFNA(FDS($C$3,"FF_COM_SHS_OUT(QTR_R,"&amp;H$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="I22" s="21">
+      <c r="I22" s="20">
         <f>_xlfn.IFNA(FDS($C$3,"FF_COM_SHS_OUT(QTR_R,"&amp;I$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="J22" s="21">
+      <c r="J22" s="20">
         <f>_xlfn.IFNA(FDS($C$3,"FF_COM_SHS_OUT(QTR_R,"&amp;J$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="K22" s="21">
+      <c r="K22" s="20">
         <f>_xlfn.IFNA(FDS($C$3,"FF_COM_SHS_OUT(QTR_R,"&amp;K$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="L22" s="21">
+      <c r="L22" s="20">
         <f>_xlfn.IFNA(FDS($C$3,"FF_COM_SHS_OUT(QTR_R,"&amp;L$5&amp;")"),"-")</f>
         <v/>
       </c>
@@ -4631,35 +4632,35 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E29" s="20">
+      <c r="E29" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_EPS(QTR_R,"&amp;E$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="F29" s="20">
+      <c r="F29" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_EPS(QTR_R,"&amp;F$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="G29" s="20">
+      <c r="G29" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_EPS(QTR_R,"&amp;G$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="H29" s="20">
+      <c r="H29" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_EPS(QTR_R,"&amp;H$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="I29" s="20">
+      <c r="I29" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_EPS(QTR_R,"&amp;I$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="J29" s="20">
+      <c r="J29" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_EPS(QTR_R,"&amp;J$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="K29" s="20">
+      <c r="K29" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_EPS(QTR_R,"&amp;K$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="L29" s="20">
+      <c r="L29" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_EPS(QTR_R,"&amp;L$5&amp;")"),"-")</f>
         <v/>
       </c>
@@ -6353,35 +6354,35 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E66" s="20">
+      <c r="E66" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_BPS_TANG(QTR,"&amp;E$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="F66" s="20">
+      <c r="F66" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_BPS_TANG(QTR,"&amp;F$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="G66" s="20">
+      <c r="G66" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_BPS_TANG(QTR,"&amp;G$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="H66" s="20">
+      <c r="H66" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_BPS_TANG(QTR,"&amp;H$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="I66" s="20">
+      <c r="I66" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_BPS_TANG(QTR,"&amp;I$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="J66" s="20">
+      <c r="J66" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_BPS_TANG(QTR,"&amp;J$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="K66" s="20">
+      <c r="K66" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_BPS_TANG(QTR,"&amp;K$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="L66" s="20">
+      <c r="L66" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FF_BPS_TANG(QTR,"&amp;L$5&amp;")"),"-")</f>
         <v/>
       </c>
@@ -6707,35 +6708,35 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E75" s="22">
+      <c r="E75" s="21">
         <f>_xlfn.IFNA(FDS($C$3,"FB_DOM_OFFCE_NUM(QTR,"&amp;E$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="F75" s="22">
+      <c r="F75" s="21">
         <f>_xlfn.IFNA(FDS($C$3,"FB_DOM_OFFCE_NUM(QTR,"&amp;F$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="G75" s="22">
+      <c r="G75" s="21">
         <f>_xlfn.IFNA(FDS($C$3,"FB_DOM_OFFCE_NUM(QTR,"&amp;G$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="H75" s="22">
+      <c r="H75" s="21">
         <f>_xlfn.IFNA(FDS($C$3,"FB_DOM_OFFCE_NUM(QTR,"&amp;H$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="I75" s="22">
+      <c r="I75" s="21">
         <f>_xlfn.IFNA(FDS($C$3,"FB_DOM_OFFCE_NUM(QTR,"&amp;I$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="J75" s="22">
+      <c r="J75" s="21">
         <f>_xlfn.IFNA(FDS($C$3,"FB_DOM_OFFCE_NUM(QTR,"&amp;J$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="K75" s="22">
+      <c r="K75" s="21">
         <f>_xlfn.IFNA(FDS($C$3,"FB_DOM_OFFCE_NUM(QTR,"&amp;K$5&amp;")"),"-")</f>
         <v/>
       </c>
-      <c r="L75" s="22">
+      <c r="L75" s="21">
         <f>_xlfn.IFNA(FDS($C$3,"FB_DOM_OFFCE_NUM(QTR,"&amp;L$5&amp;")"),"-")</f>
         <v/>
       </c>
@@ -6775,35 +6776,35 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E77" s="20">
+      <c r="E77" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FE_ESTIMATE(EPS_NONGAAP,MEAN,QTR,"&amp;E$5&amp;",0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="F77" s="20">
+      <c r="F77" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FE_ESTIMATE(EPS_NONGAAP,MEAN,QTR,"&amp;F$5&amp;",0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="G77" s="20">
+      <c r="G77" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FE_ESTIMATE(EPS_NONGAAP,MEAN,QTR,"&amp;G$5&amp;",0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="H77" s="20">
+      <c r="H77" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FE_ESTIMATE(EPS_NONGAAP,MEAN,QTR,"&amp;H$5&amp;",0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="I77" s="20">
+      <c r="I77" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FE_ESTIMATE(EPS_NONGAAP,MEAN,QTR,"&amp;I$5&amp;",0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="J77" s="20">
+      <c r="J77" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FE_ESTIMATE(EPS_NONGAAP,MEAN,QTR,"&amp;J$5&amp;",0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="K77" s="20">
+      <c r="K77" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FE_ESTIMATE(EPS_NONGAAP,MEAN,QTR,"&amp;K$5&amp;",0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="L77" s="20">
+      <c r="L77" s="19">
         <f>_xlfn.IFNA(FDS($C$3,"FE_ESTIMATE(EPS_NONGAAP,MEAN,QTR,"&amp;L$5&amp;",0,,,'')"),"-")</f>
         <v/>
       </c>
@@ -7099,7 +7100,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Each metric is pulled four ways: FFI_, FF_, FB_ (US banks only) and the FFI@FF@FB chain. This shows which family works per bank and whether the cross-family chain fills in. $ in millions USD; % as whole numbers.</t>
+          <t>Each metric is pulled four ways: FFI_, FF_, FB_ (US banks only) and the FFI@FF@FB chain. This shows which family works per bank; the chain takes the first one that returns a number. $ in millions USD; % as whole numbers.</t>
         </is>
       </c>
     </row>
@@ -7277,9 +7278,9 @@
           <t>FF_BK_COM_EQ_TIER1_TOT(ANN_R,{y},,,,USD)</t>
         </is>
       </c>
-      <c r="D10" s="25" t="inlineStr">
-        <is>
-          <t>Not in catalog</t>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E10" s="17">
@@ -7319,9 +7320,9 @@
           <t>FB_COM_EQ_TIER1(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E11" s="17">
@@ -7361,32 +7362,32 @@
           <t>FFI_COM_EQ_TIER1_TOT(ANN_L,{y},,,,USD)@FF_BK_COM_EQ_TIER1_TOT(ANN_R,{y},,,,USD)@FB_COM_EQ_TIER1(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E12" s="26">
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E12" s="25">
         <f>FDSC("-",E$6,"FFI_COM_EQ_TIER1_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_BK_COM_EQ_TIER1_TOT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_COM_EQ_TIER1(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="F12" s="26">
+      <c r="F12" s="25">
         <f>FDSC("-",F$6,"FFI_COM_EQ_TIER1_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_BK_COM_EQ_TIER1_TOT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_COM_EQ_TIER1(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="G12" s="26">
+      <c r="G12" s="25">
         <f>FDSC("-",G$6,"FFI_COM_EQ_TIER1_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_BK_COM_EQ_TIER1_TOT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_COM_EQ_TIER1(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="H12" s="26">
+      <c r="H12" s="25">
         <f>FDSC("-",H$6,"FFI_COM_EQ_TIER1_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_BK_COM_EQ_TIER1_TOT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_COM_EQ_TIER1(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="I12" s="26">
+      <c r="I12" s="25">
         <f>FDSC("-",I$6,"FFI_COM_EQ_TIER1_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_BK_COM_EQ_TIER1_TOT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_COM_EQ_TIER1(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="J12" s="26">
+      <c r="J12" s="25">
         <f>FDSC("-",J$6,"FFI_COM_EQ_TIER1_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_BK_COM_EQ_TIER1_TOT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_COM_EQ_TIER1(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
@@ -7529,32 +7530,32 @@
           <t>FFI_COM_EQ_TIER1_RATIO(ANN_L,{y})@FF_BK_COM_EQ_TIER1_RATIO(ANN_R,{y})@FB_COM_EQ_TIER1_RATIO(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E16" s="27">
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E16" s="26">
         <f>FDSC("-",E$6,"FFI_COM_EQ_TIER1_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_COM_EQ_TIER1_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_COM_EQ_TIER1_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="F16" s="27">
+      <c r="F16" s="26">
         <f>FDSC("-",F$6,"FFI_COM_EQ_TIER1_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_COM_EQ_TIER1_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_COM_EQ_TIER1_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="G16" s="27">
+      <c r="G16" s="26">
         <f>FDSC("-",G$6,"FFI_COM_EQ_TIER1_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_COM_EQ_TIER1_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_COM_EQ_TIER1_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="H16" s="27">
+      <c r="H16" s="26">
         <f>FDSC("-",H$6,"FFI_COM_EQ_TIER1_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_COM_EQ_TIER1_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_COM_EQ_TIER1_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="I16" s="27">
+      <c r="I16" s="26">
         <f>FDSC("-",I$6,"FFI_COM_EQ_TIER1_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_COM_EQ_TIER1_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_COM_EQ_TIER1_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="J16" s="27">
+      <c r="J16" s="26">
         <f>FDSC("-",J$6,"FFI_COM_EQ_TIER1_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_COM_EQ_TIER1_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_COM_EQ_TIER1_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
@@ -7613,9 +7614,9 @@
           <t>FF_TIER1_CAP(ANN_R,{y},,,,USD)</t>
         </is>
       </c>
-      <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E18" s="17">
@@ -7655,9 +7656,9 @@
           <t>FB_TIER1_CAP(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E19" s="17">
@@ -7697,32 +7698,32 @@
           <t>FFI_TIER1_CAP(ANN_L,{y},,,,USD)@FF_TIER1_CAP(ANN_R,{y},,,,USD)@FB_TIER1_CAP(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E20" s="26">
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E20" s="25">
         <f>FDSC("-",E$6,"FFI_TIER1_CAP(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_TIER1_CAP(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_TIER1_CAP(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="F20" s="26">
+      <c r="F20" s="25">
         <f>FDSC("-",F$6,"FFI_TIER1_CAP(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_TIER1_CAP(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_TIER1_CAP(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="G20" s="26">
+      <c r="G20" s="25">
         <f>FDSC("-",G$6,"FFI_TIER1_CAP(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_TIER1_CAP(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_TIER1_CAP(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="H20" s="26">
+      <c r="H20" s="25">
         <f>FDSC("-",H$6,"FFI_TIER1_CAP(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_TIER1_CAP(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_TIER1_CAP(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="I20" s="26">
+      <c r="I20" s="25">
         <f>FDSC("-",I$6,"FFI_TIER1_CAP(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_TIER1_CAP(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_TIER1_CAP(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="J20" s="26">
+      <c r="J20" s="25">
         <f>FDSC("-",J$6,"FFI_TIER1_CAP(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_TIER1_CAP(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_TIER1_CAP(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
@@ -7781,9 +7782,9 @@
           <t>FF_CAP_RATIO_TIER1(ANN_R,{y})</t>
         </is>
       </c>
-      <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E22" s="18">
@@ -7823,9 +7824,9 @@
           <t>FB_CAP_RATIO_TIER1(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D23" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E23" s="18">
@@ -7865,32 +7866,32 @@
           <t>FFI_CAP_RATIO_TIER1(ANN_L,{y})@FF_CAP_RATIO_TIER1(ANN_R,{y})@FB_CAP_RATIO_TIER1(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D24" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E24" s="27">
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E24" s="26">
         <f>FDSC("-",E$6,"FFI_CAP_RATIO_TIER1(ANN_L,"&amp;$C$3&amp;")@FF_CAP_RATIO_TIER1(ANN_R,"&amp;$C$3&amp;")@FB_CAP_RATIO_TIER1(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="F24" s="27">
+      <c r="F24" s="26">
         <f>FDSC("-",F$6,"FFI_CAP_RATIO_TIER1(ANN_L,"&amp;$C$3&amp;")@FF_CAP_RATIO_TIER1(ANN_R,"&amp;$C$3&amp;")@FB_CAP_RATIO_TIER1(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="G24" s="27">
+      <c r="G24" s="26">
         <f>FDSC("-",G$6,"FFI_CAP_RATIO_TIER1(ANN_L,"&amp;$C$3&amp;")@FF_CAP_RATIO_TIER1(ANN_R,"&amp;$C$3&amp;")@FB_CAP_RATIO_TIER1(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="H24" s="27">
+      <c r="H24" s="26">
         <f>FDSC("-",H$6,"FFI_CAP_RATIO_TIER1(ANN_L,"&amp;$C$3&amp;")@FF_CAP_RATIO_TIER1(ANN_R,"&amp;$C$3&amp;")@FB_CAP_RATIO_TIER1(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="I24" s="27">
+      <c r="I24" s="26">
         <f>FDSC("-",I$6,"FFI_CAP_RATIO_TIER1(ANN_L,"&amp;$C$3&amp;")@FF_CAP_RATIO_TIER1(ANN_R,"&amp;$C$3&amp;")@FB_CAP_RATIO_TIER1(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="J24" s="27">
+      <c r="J24" s="26">
         <f>FDSC("-",J$6,"FFI_CAP_RATIO_TIER1(ANN_L,"&amp;$C$3&amp;")@FF_CAP_RATIO_TIER1(ANN_R,"&amp;$C$3&amp;")@FB_CAP_RATIO_TIER1(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
@@ -7949,9 +7950,9 @@
           <t>FF_CAP_RATIO_TOT(ANN_R,{y})</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E26" s="18">
@@ -7991,9 +7992,9 @@
           <t>FB_CAP_RATIO_TOT(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D27" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E27" s="18">
@@ -8033,32 +8034,32 @@
           <t>FFI_CAP_RATIO_TOT(ANN_L,{y})@FF_CAP_RATIO_TOT(ANN_R,{y})@FB_CAP_RATIO_TOT(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D28" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E28" s="27">
+      <c r="D28" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E28" s="26">
         <f>FDSC("-",E$6,"FFI_CAP_RATIO_TOT(ANN_L,"&amp;$C$3&amp;")@FF_CAP_RATIO_TOT(ANN_R,"&amp;$C$3&amp;")@FB_CAP_RATIO_TOT(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="F28" s="27">
+      <c r="F28" s="26">
         <f>FDSC("-",F$6,"FFI_CAP_RATIO_TOT(ANN_L,"&amp;$C$3&amp;")@FF_CAP_RATIO_TOT(ANN_R,"&amp;$C$3&amp;")@FB_CAP_RATIO_TOT(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="G28" s="27">
+      <c r="G28" s="26">
         <f>FDSC("-",G$6,"FFI_CAP_RATIO_TOT(ANN_L,"&amp;$C$3&amp;")@FF_CAP_RATIO_TOT(ANN_R,"&amp;$C$3&amp;")@FB_CAP_RATIO_TOT(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="H28" s="27">
+      <c r="H28" s="26">
         <f>FDSC("-",H$6,"FFI_CAP_RATIO_TOT(ANN_L,"&amp;$C$3&amp;")@FF_CAP_RATIO_TOT(ANN_R,"&amp;$C$3&amp;")@FB_CAP_RATIO_TOT(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="I28" s="27">
+      <c r="I28" s="26">
         <f>FDSC("-",I$6,"FFI_CAP_RATIO_TOT(ANN_L,"&amp;$C$3&amp;")@FF_CAP_RATIO_TOT(ANN_R,"&amp;$C$3&amp;")@FB_CAP_RATIO_TOT(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="J28" s="27">
+      <c r="J28" s="26">
         <f>FDSC("-",J$6,"FFI_CAP_RATIO_TOT(ANN_L,"&amp;$C$3&amp;")@FF_CAP_RATIO_TOT(ANN_R,"&amp;$C$3&amp;")@FB_CAP_RATIO_TOT(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
@@ -8075,9 +8076,9 @@
           <t>FFI_LEV_RATIO_RPT(ANN_L,{y})</t>
         </is>
       </c>
-      <c r="D29" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E29" s="18">
@@ -8159,9 +8160,9 @@
           <t>FB_LEV_RATIO(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D31" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E31" s="18">
@@ -8201,32 +8202,32 @@
           <t>FFI_LEV_RATIO_RPT(ANN_L,{y})@FF_BK_LEV_RATIO(ANN_R,{y})@FB_LEV_RATIO(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D32" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E32" s="27">
+      <c r="D32" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E32" s="26">
         <f>FDSC("-",E$6,"FFI_LEV_RATIO_RPT(ANN_L,"&amp;$C$3&amp;")@FF_BK_LEV_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_LEV_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="F32" s="27">
+      <c r="F32" s="26">
         <f>FDSC("-",F$6,"FFI_LEV_RATIO_RPT(ANN_L,"&amp;$C$3&amp;")@FF_BK_LEV_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_LEV_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="G32" s="27">
+      <c r="G32" s="26">
         <f>FDSC("-",G$6,"FFI_LEV_RATIO_RPT(ANN_L,"&amp;$C$3&amp;")@FF_BK_LEV_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_LEV_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="H32" s="27">
+      <c r="H32" s="26">
         <f>FDSC("-",H$6,"FFI_LEV_RATIO_RPT(ANN_L,"&amp;$C$3&amp;")@FF_BK_LEV_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_LEV_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="I32" s="27">
+      <c r="I32" s="26">
         <f>FDSC("-",I$6,"FFI_LEV_RATIO_RPT(ANN_L,"&amp;$C$3&amp;")@FF_BK_LEV_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_LEV_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="J32" s="27">
+      <c r="J32" s="26">
         <f>FDSC("-",J$6,"FFI_LEV_RATIO_RPT(ANN_L,"&amp;$C$3&amp;")@FF_BK_LEV_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_LEV_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
@@ -8327,9 +8328,9 @@
           <t>FB_ASSETS_RISK_WGHT(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D35" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E35" s="17">
@@ -8369,32 +8370,32 @@
           <t>FFI_RWA(ANN_L,{y},,,,USD)@FF_ASSETS_RISK_WGHT(ANN_R,{y},,,,USD)@FB_ASSETS_RISK_WGHT(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E36" s="26">
+      <c r="D36" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E36" s="25">
         <f>FDSC("-",E$6,"FFI_RWA(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_ASSETS_RISK_WGHT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_ASSETS_RISK_WGHT(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="F36" s="26">
+      <c r="F36" s="25">
         <f>FDSC("-",F$6,"FFI_RWA(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_ASSETS_RISK_WGHT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_ASSETS_RISK_WGHT(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="G36" s="26">
+      <c r="G36" s="25">
         <f>FDSC("-",G$6,"FFI_RWA(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_ASSETS_RISK_WGHT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_ASSETS_RISK_WGHT(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="H36" s="26">
+      <c r="H36" s="25">
         <f>FDSC("-",H$6,"FFI_RWA(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_ASSETS_RISK_WGHT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_ASSETS_RISK_WGHT(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="I36" s="26">
+      <c r="I36" s="25">
         <f>FDSC("-",I$6,"FFI_RWA(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_ASSETS_RISK_WGHT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_ASSETS_RISK_WGHT(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="J36" s="26">
+      <c r="J36" s="25">
         <f>FDSC("-",J$6,"FFI_RWA(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_ASSETS_RISK_WGHT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_ASSETS_RISK_WGHT(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
@@ -8427,9 +8428,9 @@
           <t>FFI_NPL_LOAN_ADV(ANN_L,{y},,,,USD)</t>
         </is>
       </c>
-      <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E38" s="17">
@@ -8511,9 +8512,9 @@
           <t>FB_NONPERF_LOAN(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D40" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D40" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E40" s="17">
@@ -8553,32 +8554,32 @@
           <t>FFI_NPL_LOAN_ADV(ANN_L,{y},,,,USD)@FF_LOAN_NONPERF(ANN_R,{y},,,,USD)@FB_NONPERF_LOAN(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D41" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E41" s="26">
+      <c r="D41" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E41" s="25">
         <f>FDSC("-",E$6,"FFI_NPL_LOAN_ADV(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_NONPERF(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_NONPERF_LOAN(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="F41" s="26">
+      <c r="F41" s="25">
         <f>FDSC("-",F$6,"FFI_NPL_LOAN_ADV(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_NONPERF(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_NONPERF_LOAN(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="G41" s="26">
+      <c r="G41" s="25">
         <f>FDSC("-",G$6,"FFI_NPL_LOAN_ADV(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_NONPERF(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_NONPERF_LOAN(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="H41" s="26">
+      <c r="H41" s="25">
         <f>FDSC("-",H$6,"FFI_NPL_LOAN_ADV(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_NONPERF(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_NONPERF_LOAN(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="I41" s="26">
+      <c r="I41" s="25">
         <f>FDSC("-",I$6,"FFI_NPL_LOAN_ADV(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_NONPERF(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_NONPERF_LOAN(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="J41" s="26">
+      <c r="J41" s="25">
         <f>FDSC("-",J$6,"FFI_NPL_LOAN_ADV(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_NONPERF(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_NONPERF_LOAN(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
@@ -8595,9 +8596,9 @@
           <t>FFI_LOAN_LOSS_PROV(ANN_L,{y},,,,USD)</t>
         </is>
       </c>
-      <c r="D42" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E42" s="17">
@@ -8679,9 +8680,9 @@
           <t>FB_LOAN_LOSS_PROV(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D44" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E44" s="17">
@@ -8721,32 +8722,32 @@
           <t>FFI_LOAN_LOSS_PROV(ANN_L,{y},,,,USD)@FF_LOAN_LOSS_PROV(ANN_R,{y},,,,USD)@FB_LOAN_LOSS_PROV(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D45" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E45" s="26">
+      <c r="D45" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E45" s="25">
         <f>FDSC("-",E$6,"FFI_LOAN_LOSS_PROV(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_LOSS_PROV(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_LOAN_LOSS_PROV(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="F45" s="26">
+      <c r="F45" s="25">
         <f>FDSC("-",F$6,"FFI_LOAN_LOSS_PROV(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_LOSS_PROV(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_LOAN_LOSS_PROV(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="G45" s="26">
+      <c r="G45" s="25">
         <f>FDSC("-",G$6,"FFI_LOAN_LOSS_PROV(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_LOSS_PROV(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_LOAN_LOSS_PROV(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="H45" s="26">
+      <c r="H45" s="25">
         <f>FDSC("-",H$6,"FFI_LOAN_LOSS_PROV(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_LOSS_PROV(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_LOAN_LOSS_PROV(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="I45" s="26">
+      <c r="I45" s="25">
         <f>FDSC("-",I$6,"FFI_LOAN_LOSS_PROV(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_LOSS_PROV(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_LOAN_LOSS_PROV(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="J45" s="26">
+      <c r="J45" s="25">
         <f>FDSC("-",J$6,"FFI_LOAN_LOSS_PROV(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_LOSS_PROV(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_LOAN_LOSS_PROV(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
@@ -8805,9 +8806,9 @@
           <t>FFI_NPL_LOAN_LOSS_RSRV_RATIO(ANN_L,{y})</t>
         </is>
       </c>
-      <c r="D47" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D47" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E47" s="18">
@@ -8847,9 +8848,9 @@
           <t>FF_NONPERF_LOAN_LOSS_RSRV(ANN_R,{y})</t>
         </is>
       </c>
-      <c r="D48" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E48" s="18">
@@ -8889,32 +8890,32 @@
           <t>FFI_NPL_LOAN_LOSS_RSRV_RATIO(ANN_L,{y})@FF_NONPERF_LOAN_LOSS_RSRV(ANN_R,{y})</t>
         </is>
       </c>
-      <c r="D49" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E49" s="27">
+      <c r="D49" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E49" s="26">
         <f>FDSC("-",E$6,"FFI_NPL_LOAN_LOSS_RSRV_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_NONPERF_LOAN_LOSS_RSRV(ANN_R,"&amp;$C$3&amp;")")</f>
         <v/>
       </c>
-      <c r="F49" s="27">
+      <c r="F49" s="26">
         <f>FDSC("-",F$6,"FFI_NPL_LOAN_LOSS_RSRV_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_NONPERF_LOAN_LOSS_RSRV(ANN_R,"&amp;$C$3&amp;")")</f>
         <v/>
       </c>
-      <c r="G49" s="27">
+      <c r="G49" s="26">
         <f>FDSC("-",G$6,"FFI_NPL_LOAN_LOSS_RSRV_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_NONPERF_LOAN_LOSS_RSRV(ANN_R,"&amp;$C$3&amp;")")</f>
         <v/>
       </c>
-      <c r="H49" s="27">
+      <c r="H49" s="26">
         <f>FDSC("-",H$6,"FFI_NPL_LOAN_LOSS_RSRV_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_NONPERF_LOAN_LOSS_RSRV(ANN_R,"&amp;$C$3&amp;")")</f>
         <v/>
       </c>
-      <c r="I49" s="27">
+      <c r="I49" s="26">
         <f>FDSC("-",I$6,"FFI_NPL_LOAN_LOSS_RSRV_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_NONPERF_LOAN_LOSS_RSRV(ANN_R,"&amp;$C$3&amp;")")</f>
         <v/>
       </c>
-      <c r="J49" s="27">
+      <c r="J49" s="26">
         <f>FDSC("-",J$6,"FFI_NPL_LOAN_LOSS_RSRV_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_NONPERF_LOAN_LOSS_RSRV(ANN_R,"&amp;$C$3&amp;")")</f>
         <v/>
       </c>
@@ -8931,9 +8932,9 @@
           <t>FFI_NPL_LOAN_RATIO(ANN_L,{y})</t>
         </is>
       </c>
-      <c r="D50" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E50" s="18">
@@ -9015,9 +9016,9 @@
           <t>FB_NONPERF_LOAN_PCT(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D52" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E52" s="18">
@@ -9057,32 +9058,32 @@
           <t>FFI_NPL_LOAN_RATIO(ANN_L,{y})@FF_NONPERF_LOAN_PCT(ANN_R,{y})@FB_NONPERF_LOAN_PCT(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D53" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E53" s="27">
+      <c r="D53" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E53" s="26">
         <f>FDSC("-",E$6,"FFI_NPL_LOAN_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_NONPERF_LOAN_PCT(ANN_R,"&amp;$C$3&amp;")@FB_NONPERF_LOAN_PCT(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="F53" s="27">
+      <c r="F53" s="26">
         <f>FDSC("-",F$6,"FFI_NPL_LOAN_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_NONPERF_LOAN_PCT(ANN_R,"&amp;$C$3&amp;")@FB_NONPERF_LOAN_PCT(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="G53" s="27">
+      <c r="G53" s="26">
         <f>FDSC("-",G$6,"FFI_NPL_LOAN_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_NONPERF_LOAN_PCT(ANN_R,"&amp;$C$3&amp;")@FB_NONPERF_LOAN_PCT(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="H53" s="27">
+      <c r="H53" s="26">
         <f>FDSC("-",H$6,"FFI_NPL_LOAN_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_NONPERF_LOAN_PCT(ANN_R,"&amp;$C$3&amp;")@FB_NONPERF_LOAN_PCT(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="I53" s="27">
+      <c r="I53" s="26">
         <f>FDSC("-",I$6,"FFI_NPL_LOAN_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_NONPERF_LOAN_PCT(ANN_R,"&amp;$C$3&amp;")@FB_NONPERF_LOAN_PCT(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="J53" s="27">
+      <c r="J53" s="26">
         <f>FDSC("-",J$6,"FFI_NPL_LOAN_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_NONPERF_LOAN_PCT(ANN_R,"&amp;$C$3&amp;")@FB_NONPERF_LOAN_PCT(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
@@ -9199,9 +9200,9 @@
           <t>FB_EFF_RATIO(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D57" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D57" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E57" s="18">
@@ -9241,32 +9242,32 @@
           <t>FFI_EFF_RATIO(ANN_L,{y})@FF_BK_EFF_RATIO(ANN_R,{y})@FB_EFF_RATIO(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D58" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E58" s="27">
+      <c r="D58" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E58" s="26">
         <f>FDSC("-",E$6,"FFI_EFF_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_EFF_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_EFF_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="F58" s="27">
+      <c r="F58" s="26">
         <f>FDSC("-",F$6,"FFI_EFF_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_EFF_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_EFF_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="G58" s="27">
+      <c r="G58" s="26">
         <f>FDSC("-",G$6,"FFI_EFF_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_EFF_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_EFF_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="H58" s="27">
+      <c r="H58" s="26">
         <f>FDSC("-",H$6,"FFI_EFF_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_EFF_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_EFF_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="I58" s="27">
+      <c r="I58" s="26">
         <f>FDSC("-",I$6,"FFI_EFF_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_EFF_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_EFF_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="J58" s="27">
+      <c r="J58" s="26">
         <f>FDSC("-",J$6,"FFI_EFF_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_EFF_RATIO(ANN_R,"&amp;$C$3&amp;")@FB_EFF_RATIO(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
@@ -9341,9 +9342,9 @@
           <t>FB_ROTE(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D61" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E61" s="18">
@@ -9383,32 +9384,32 @@
           <t>FFI_ROTE(ANN_L,{y})@FB_ROTE(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D62" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E62" s="27">
+      <c r="D62" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E62" s="26">
         <f>FDSC("-",E$6,"FFI_ROTE(ANN_L,"&amp;$C$3&amp;")@FB_ROTE(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="F62" s="27">
+      <c r="F62" s="26">
         <f>FDSC("-",F$6,"FFI_ROTE(ANN_L,"&amp;$C$3&amp;")@FB_ROTE(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="G62" s="27">
+      <c r="G62" s="26">
         <f>FDSC("-",G$6,"FFI_ROTE(ANN_L,"&amp;$C$3&amp;")@FB_ROTE(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="H62" s="27">
+      <c r="H62" s="26">
         <f>FDSC("-",H$6,"FFI_ROTE(ANN_L,"&amp;$C$3&amp;")@FB_ROTE(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="I62" s="27">
+      <c r="I62" s="26">
         <f>FDSC("-",I$6,"FFI_ROTE(ANN_L,"&amp;$C$3&amp;")@FB_ROTE(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="J62" s="27">
+      <c r="J62" s="26">
         <f>FDSC("-",J$6,"FFI_ROTE(ANN_L,"&amp;$C$3&amp;")@FB_ROTE(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
@@ -9551,32 +9552,32 @@
           <t>FFI_ROTCE(ANN_L,{y})@FF_ROTCE(ANN_R,{y})@FB_ROTCE(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D66" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E66" s="27">
+      <c r="D66" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E66" s="26">
         <f>FDSC("-",E$6,"FFI_ROTCE(ANN_L,"&amp;$C$3&amp;")@FF_ROTCE(ANN_R,"&amp;$C$3&amp;")@FB_ROTCE(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="F66" s="27">
+      <c r="F66" s="26">
         <f>FDSC("-",F$6,"FFI_ROTCE(ANN_L,"&amp;$C$3&amp;")@FF_ROTCE(ANN_R,"&amp;$C$3&amp;")@FB_ROTCE(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="G66" s="27">
+      <c r="G66" s="26">
         <f>FDSC("-",G$6,"FFI_ROTCE(ANN_L,"&amp;$C$3&amp;")@FF_ROTCE(ANN_R,"&amp;$C$3&amp;")@FB_ROTCE(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="H66" s="27">
+      <c r="H66" s="26">
         <f>FDSC("-",H$6,"FFI_ROTCE(ANN_L,"&amp;$C$3&amp;")@FF_ROTCE(ANN_R,"&amp;$C$3&amp;")@FB_ROTCE(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="I66" s="27">
+      <c r="I66" s="26">
         <f>FDSC("-",I$6,"FFI_ROTCE(ANN_L,"&amp;$C$3&amp;")@FF_ROTCE(ANN_R,"&amp;$C$3&amp;")@FB_ROTCE(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="J66" s="27">
+      <c r="J66" s="26">
         <f>FDSC("-",J$6,"FFI_ROTCE(ANN_L,"&amp;$C$3&amp;")@FF_ROTCE(ANN_R,"&amp;$C$3&amp;")@FB_ROTCE(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
@@ -9677,9 +9678,9 @@
           <t>FB_ROA(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D69" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D69" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E69" s="18">
@@ -9719,32 +9720,32 @@
           <t>FFI_ROA(ANN_L,{y})@FF_ROA(ANN_R,{y})@FB_ROA(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D70" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E70" s="27">
+      <c r="D70" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E70" s="26">
         <f>FDSC("-",E$6,"FFI_ROA(ANN_L,"&amp;$C$3&amp;")@FF_ROA(ANN_R,"&amp;$C$3&amp;")@FB_ROA(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="F70" s="27">
+      <c r="F70" s="26">
         <f>FDSC("-",F$6,"FFI_ROA(ANN_L,"&amp;$C$3&amp;")@FF_ROA(ANN_R,"&amp;$C$3&amp;")@FB_ROA(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="G70" s="27">
+      <c r="G70" s="26">
         <f>FDSC("-",G$6,"FFI_ROA(ANN_L,"&amp;$C$3&amp;")@FF_ROA(ANN_R,"&amp;$C$3&amp;")@FB_ROA(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="H70" s="27">
+      <c r="H70" s="26">
         <f>FDSC("-",H$6,"FFI_ROA(ANN_L,"&amp;$C$3&amp;")@FF_ROA(ANN_R,"&amp;$C$3&amp;")@FB_ROA(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="I70" s="27">
+      <c r="I70" s="26">
         <f>FDSC("-",I$6,"FFI_ROA(ANN_L,"&amp;$C$3&amp;")@FF_ROA(ANN_R,"&amp;$C$3&amp;")@FB_ROA(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="J70" s="27">
+      <c r="J70" s="26">
         <f>FDSC("-",J$6,"FFI_ROA(ANN_L,"&amp;$C$3&amp;")@FF_ROA(ANN_R,"&amp;$C$3&amp;")@FB_ROA(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
@@ -9761,9 +9762,9 @@
           <t>FFI_AVG_BAL_INT_RATE_NET_MGN(ANN_L,{y})</t>
         </is>
       </c>
-      <c r="D71" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D71" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E71" s="18">
@@ -9887,32 +9888,32 @@
           <t>FFI_AVG_BAL_INT_RATE_NET_MGN(ANN_L,{y})@FF_INT_MGN(ANN_R,{y})@FB_INT_MGN(ANN,{y},,,RF)</t>
         </is>
       </c>
-      <c r="D74" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E74" s="27">
+      <c r="D74" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E74" s="26">
         <f>FDSC("-",E$6,"FFI_AVG_BAL_INT_RATE_NET_MGN(ANN_L,"&amp;$C$3&amp;")@FF_INT_MGN(ANN_R,"&amp;$C$3&amp;")@FB_INT_MGN(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="F74" s="27">
+      <c r="F74" s="26">
         <f>FDSC("-",F$6,"FFI_AVG_BAL_INT_RATE_NET_MGN(ANN_L,"&amp;$C$3&amp;")@FF_INT_MGN(ANN_R,"&amp;$C$3&amp;")@FB_INT_MGN(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="G74" s="27">
+      <c r="G74" s="26">
         <f>FDSC("-",G$6,"FFI_AVG_BAL_INT_RATE_NET_MGN(ANN_L,"&amp;$C$3&amp;")@FF_INT_MGN(ANN_R,"&amp;$C$3&amp;")@FB_INT_MGN(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="H74" s="27">
+      <c r="H74" s="26">
         <f>FDSC("-",H$6,"FFI_AVG_BAL_INT_RATE_NET_MGN(ANN_L,"&amp;$C$3&amp;")@FF_INT_MGN(ANN_R,"&amp;$C$3&amp;")@FB_INT_MGN(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="I74" s="27">
+      <c r="I74" s="26">
         <f>FDSC("-",I$6,"FFI_AVG_BAL_INT_RATE_NET_MGN(ANN_L,"&amp;$C$3&amp;")@FF_INT_MGN(ANN_R,"&amp;$C$3&amp;")@FB_INT_MGN(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
-      <c r="J74" s="27">
+      <c r="J74" s="26">
         <f>FDSC("-",J$6,"FFI_AVG_BAL_INT_RATE_NET_MGN(ANN_L,"&amp;$C$3&amp;")@FF_INT_MGN(ANN_R,"&amp;$C$3&amp;")@FB_INT_MGN(ANN,"&amp;$C$3&amp;",,,RF)")</f>
         <v/>
       </c>
@@ -10013,9 +10014,9 @@
           <t>FB_INT_INC_NET(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D77" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D77" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E77" s="17">
@@ -10055,32 +10056,32 @@
           <t>FFI_INT_INC_NET(ANN_L,{y},,,,USD)@FF_INT_INC_NET(ANN_R,{y},,,,USD)@FB_INT_INC_NET(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D78" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E78" s="26">
+      <c r="D78" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E78" s="25">
         <f>FDSC("-",E$6,"FFI_INT_INC_NET(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_INT_INC_NET(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_INT_INC_NET(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="F78" s="26">
+      <c r="F78" s="25">
         <f>FDSC("-",F$6,"FFI_INT_INC_NET(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_INT_INC_NET(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_INT_INC_NET(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="G78" s="26">
+      <c r="G78" s="25">
         <f>FDSC("-",G$6,"FFI_INT_INC_NET(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_INT_INC_NET(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_INT_INC_NET(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="H78" s="26">
+      <c r="H78" s="25">
         <f>FDSC("-",H$6,"FFI_INT_INC_NET(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_INT_INC_NET(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_INT_INC_NET(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="I78" s="26">
+      <c r="I78" s="25">
         <f>FDSC("-",I$6,"FFI_INT_INC_NET(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_INT_INC_NET(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_INT_INC_NET(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="J78" s="26">
+      <c r="J78" s="25">
         <f>FDSC("-",J$6,"FFI_INT_INC_NET(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_INT_INC_NET(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_INT_INC_NET(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
@@ -10181,9 +10182,9 @@
           <t>FB_NON_INT_INC(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D81" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D81" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E81" s="17">
@@ -10223,32 +10224,32 @@
           <t>FFI_NON_INT_INC(ANN_L,{y},,,,USD)@FF_NON_INT_INC(ANN_R,{y},,,,USD)@FB_NON_INT_INC(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D82" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E82" s="26">
+      <c r="D82" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E82" s="25">
         <f>FDSC("-",E$6,"FFI_NON_INT_INC(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_NON_INT_INC(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_NON_INT_INC(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="F82" s="26">
+      <c r="F82" s="25">
         <f>FDSC("-",F$6,"FFI_NON_INT_INC(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_NON_INT_INC(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_NON_INT_INC(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="G82" s="26">
+      <c r="G82" s="25">
         <f>FDSC("-",G$6,"FFI_NON_INT_INC(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_NON_INT_INC(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_NON_INT_INC(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="H82" s="26">
+      <c r="H82" s="25">
         <f>FDSC("-",H$6,"FFI_NON_INT_INC(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_NON_INT_INC(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_NON_INT_INC(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="I82" s="26">
+      <c r="I82" s="25">
         <f>FDSC("-",I$6,"FFI_NON_INT_INC(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_NON_INT_INC(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_NON_INT_INC(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="J82" s="26">
+      <c r="J82" s="25">
         <f>FDSC("-",J$6,"FFI_NON_INT_INC(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_NON_INT_INC(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_NON_INT_INC(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
@@ -10365,9 +10366,9 @@
           <t>FB_TOT_HFI_HFS_UNEARN_INC(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D86" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D86" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E86" s="17">
@@ -10407,32 +10408,32 @@
           <t>FFI_LOAN_ADV_TOT(ANN_L,{y},,,,USD)@FF_BK_LOAN_TOT(ANN_R,{y},,,,USD)@FB_TOT_HFI_HFS_UNEARN_INC(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D87" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E87" s="26">
+      <c r="D87" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E87" s="25">
         <f>FDSC("-",E$6,"FFI_LOAN_ADV_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_BK_LOAN_TOT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_TOT_HFI_HFS_UNEARN_INC(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="F87" s="26">
+      <c r="F87" s="25">
         <f>FDSC("-",F$6,"FFI_LOAN_ADV_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_BK_LOAN_TOT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_TOT_HFI_HFS_UNEARN_INC(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="G87" s="26">
+      <c r="G87" s="25">
         <f>FDSC("-",G$6,"FFI_LOAN_ADV_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_BK_LOAN_TOT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_TOT_HFI_HFS_UNEARN_INC(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="H87" s="26">
+      <c r="H87" s="25">
         <f>FDSC("-",H$6,"FFI_LOAN_ADV_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_BK_LOAN_TOT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_TOT_HFI_HFS_UNEARN_INC(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="I87" s="26">
+      <c r="I87" s="25">
         <f>FDSC("-",I$6,"FFI_LOAN_ADV_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_BK_LOAN_TOT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_TOT_HFI_HFS_UNEARN_INC(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="J87" s="26">
+      <c r="J87" s="25">
         <f>FDSC("-",J$6,"FFI_LOAN_ADV_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_BK_LOAN_TOT(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_TOT_HFI_HFS_UNEARN_INC(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
@@ -10533,9 +10534,9 @@
           <t>FB_DEPS(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D90" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D90" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E90" s="17">
@@ -10575,32 +10576,32 @@
           <t>FFI_DEPS_TOT(ANN_L,{y},,,,USD)@FF_DEPS(ANN_R,{y},,,,USD)@FB_DEPS(ANN,{y},,,RF,USD)</t>
         </is>
       </c>
-      <c r="D91" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E91" s="26">
+      <c r="D91" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E91" s="25">
         <f>FDSC("-",E$6,"FFI_DEPS_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_DEPS(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_DEPS(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="F91" s="26">
+      <c r="F91" s="25">
         <f>FDSC("-",F$6,"FFI_DEPS_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_DEPS(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_DEPS(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="G91" s="26">
+      <c r="G91" s="25">
         <f>FDSC("-",G$6,"FFI_DEPS_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_DEPS(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_DEPS(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="H91" s="26">
+      <c r="H91" s="25">
         <f>FDSC("-",H$6,"FFI_DEPS_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_DEPS(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_DEPS(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="I91" s="26">
+      <c r="I91" s="25">
         <f>FDSC("-",I$6,"FFI_DEPS_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_DEPS(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_DEPS(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
-      <c r="J91" s="26">
+      <c r="J91" s="25">
         <f>FDSC("-",J$6,"FFI_DEPS_TOT(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_DEPS(ANN_R,"&amp;$C$3&amp;",,,,USD)@FB_DEPS(ANN,"&amp;$C$3&amp;",,,RF,USD)")</f>
         <v/>
       </c>
@@ -10701,32 +10702,32 @@
           <t>FFI_BK_LIQ_COVG_RATIO(ANN_L,{y})@FF_BK_LIQ_COVG_RATIO(ANN_R,{y})</t>
         </is>
       </c>
-      <c r="D94" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E94" s="27">
+      <c r="D94" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E94" s="26">
         <f>FDSC("-",E$6,"FFI_BK_LIQ_COVG_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_LIQ_COVG_RATIO(ANN_R,"&amp;$C$3&amp;")")</f>
         <v/>
       </c>
-      <c r="F94" s="27">
+      <c r="F94" s="26">
         <f>FDSC("-",F$6,"FFI_BK_LIQ_COVG_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_LIQ_COVG_RATIO(ANN_R,"&amp;$C$3&amp;")")</f>
         <v/>
       </c>
-      <c r="G94" s="27">
+      <c r="G94" s="26">
         <f>FDSC("-",G$6,"FFI_BK_LIQ_COVG_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_LIQ_COVG_RATIO(ANN_R,"&amp;$C$3&amp;")")</f>
         <v/>
       </c>
-      <c r="H94" s="27">
+      <c r="H94" s="26">
         <f>FDSC("-",H$6,"FFI_BK_LIQ_COVG_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_LIQ_COVG_RATIO(ANN_R,"&amp;$C$3&amp;")")</f>
         <v/>
       </c>
-      <c r="I94" s="27">
+      <c r="I94" s="26">
         <f>FDSC("-",I$6,"FFI_BK_LIQ_COVG_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_LIQ_COVG_RATIO(ANN_R,"&amp;$C$3&amp;")")</f>
         <v/>
       </c>
-      <c r="J94" s="27">
+      <c r="J94" s="26">
         <f>FDSC("-",J$6,"FFI_BK_LIQ_COVG_RATIO(ANN_L,"&amp;$C$3&amp;")@FF_BK_LIQ_COVG_RATIO(ANN_R,"&amp;$C$3&amp;")")</f>
         <v/>
       </c>
@@ -10885,32 +10886,32 @@
           <t>FFI_LOAN_AMORT_CUST(ANN_L,{y},,,,USD)@FF_LOAN_NET(ANN_R,{y},,,,USD)</t>
         </is>
       </c>
-      <c r="D99" s="19" t="inlineStr">
-        <is>
-          <t>Unproven chain</t>
-        </is>
-      </c>
-      <c r="E99" s="26">
+      <c r="D99" s="24" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="E99" s="25">
         <f>FDSC("-",E$6,"FFI_LOAN_AMORT_CUST(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_NET(ANN_R,"&amp;$C$3&amp;",,,,USD)")</f>
         <v/>
       </c>
-      <c r="F99" s="26">
+      <c r="F99" s="25">
         <f>FDSC("-",F$6,"FFI_LOAN_AMORT_CUST(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_NET(ANN_R,"&amp;$C$3&amp;",,,,USD)")</f>
         <v/>
       </c>
-      <c r="G99" s="26">
+      <c r="G99" s="25">
         <f>FDSC("-",G$6,"FFI_LOAN_AMORT_CUST(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_NET(ANN_R,"&amp;$C$3&amp;",,,,USD)")</f>
         <v/>
       </c>
-      <c r="H99" s="26">
+      <c r="H99" s="25">
         <f>FDSC("-",H$6,"FFI_LOAN_AMORT_CUST(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_NET(ANN_R,"&amp;$C$3&amp;",,,,USD)")</f>
         <v/>
       </c>
-      <c r="I99" s="26">
+      <c r="I99" s="25">
         <f>FDSC("-",I$6,"FFI_LOAN_AMORT_CUST(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_NET(ANN_R,"&amp;$C$3&amp;",,,,USD)")</f>
         <v/>
       </c>
-      <c r="J99" s="26">
+      <c r="J99" s="25">
         <f>FDSC("-",J$6,"FFI_LOAN_AMORT_CUST(ANN_L,"&amp;$C$3&amp;",,,,USD)@FF_LOAN_NET(ANN_R,"&amp;$C$3&amp;",,,,USD)")</f>
         <v/>
       </c>
@@ -11138,23 +11139,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="19">
         <f>_xlfn.IFNA(FDS(E$7,"FE_ESTIMATE(EPS,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="F10" s="20">
+      <c r="F10" s="19">
         <f>_xlfn.IFNA(FDS(F$7,"FE_ESTIMATE(EPS,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="G10" s="20">
+      <c r="G10" s="19">
         <f>_xlfn.IFNA(FDS(G$7,"FE_ESTIMATE(EPS,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="H10" s="20">
+      <c r="H10" s="19">
         <f>_xlfn.IFNA(FDS(H$7,"FE_ESTIMATE(EPS,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="I10" s="20">
+      <c r="I10" s="19">
         <f>_xlfn.IFNA(FDS(I$7,"FE_ESTIMATE(EPS,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
@@ -11746,23 +11747,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E26" s="20">
+      <c r="E26" s="19">
         <f>_xlfn.IFNA(FDS(E$7,"FE_ESTIMATE(NETDIV,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="F26" s="20">
+      <c r="F26" s="19">
         <f>_xlfn.IFNA(FDS(F$7,"FE_ESTIMATE(NETDIV,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="G26" s="20">
+      <c r="G26" s="19">
         <f>_xlfn.IFNA(FDS(G$7,"FE_ESTIMATE(NETDIV,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="H26" s="20">
+      <c r="H26" s="19">
         <f>_xlfn.IFNA(FDS(H$7,"FE_ESTIMATE(NETDIV,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="I26" s="20">
+      <c r="I26" s="19">
         <f>_xlfn.IFNA(FDS(I$7,"FE_ESTIMATE(NETDIV,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
@@ -11784,23 +11785,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E27" s="20">
+      <c r="E27" s="19">
         <f>_xlfn.IFNA(FDS(E$7,"FE_ESTIMATE(BPS_TANG,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="F27" s="20">
+      <c r="F27" s="19">
         <f>_xlfn.IFNA(FDS(F$7,"FE_ESTIMATE(BPS_TANG,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="G27" s="20">
+      <c r="G27" s="19">
         <f>_xlfn.IFNA(FDS(G$7,"FE_ESTIMATE(BPS_TANG,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="H27" s="20">
+      <c r="H27" s="19">
         <f>_xlfn.IFNA(FDS(H$7,"FE_ESTIMATE(BPS_TANG,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="I27" s="20">
+      <c r="I27" s="19">
         <f>_xlfn.IFNA(FDS(I$7,"FE_ESTIMATE(BPS_TANG,MEAN,NTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
@@ -11837,23 +11838,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E29" s="20">
+      <c r="E29" s="19">
         <f>_xlfn.IFNA(FDS(E$7,"FE_ESTIMATE(EPS,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="F29" s="20">
+      <c r="F29" s="19">
         <f>_xlfn.IFNA(FDS(F$7,"FE_ESTIMATE(EPS,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="G29" s="20">
+      <c r="G29" s="19">
         <f>_xlfn.IFNA(FDS(G$7,"FE_ESTIMATE(EPS,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="H29" s="20">
+      <c r="H29" s="19">
         <f>_xlfn.IFNA(FDS(H$7,"FE_ESTIMATE(EPS,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="I29" s="20">
+      <c r="I29" s="19">
         <f>_xlfn.IFNA(FDS(I$7,"FE_ESTIMATE(EPS,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
@@ -12445,23 +12446,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E45" s="20">
+      <c r="E45" s="19">
         <f>_xlfn.IFNA(FDS(E$7,"FE_ESTIMATE(NETDIV,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="F45" s="20">
+      <c r="F45" s="19">
         <f>_xlfn.IFNA(FDS(F$7,"FE_ESTIMATE(NETDIV,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="G45" s="20">
+      <c r="G45" s="19">
         <f>_xlfn.IFNA(FDS(G$7,"FE_ESTIMATE(NETDIV,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="H45" s="20">
+      <c r="H45" s="19">
         <f>_xlfn.IFNA(FDS(H$7,"FE_ESTIMATE(NETDIV,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="I45" s="20">
+      <c r="I45" s="19">
         <f>_xlfn.IFNA(FDS(I$7,"FE_ESTIMATE(NETDIV,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
@@ -12483,23 +12484,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E46" s="20">
+      <c r="E46" s="19">
         <f>_xlfn.IFNA(FDS(E$7,"FE_ESTIMATE(BPS_TANG,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="F46" s="20">
+      <c r="F46" s="19">
         <f>_xlfn.IFNA(FDS(F$7,"FE_ESTIMATE(BPS_TANG,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="G46" s="20">
+      <c r="G46" s="19">
         <f>_xlfn.IFNA(FDS(G$7,"FE_ESTIMATE(BPS_TANG,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="H46" s="20">
+      <c r="H46" s="19">
         <f>_xlfn.IFNA(FDS(H$7,"FE_ESTIMATE(BPS_TANG,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="I46" s="20">
+      <c r="I46" s="19">
         <f>_xlfn.IFNA(FDS(I$7,"FE_ESTIMATE(BPS_TANG,MEAN,ANN_ROLL,"&amp;$C$3&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
@@ -12536,23 +12537,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E48" s="20">
+      <c r="E48" s="19">
         <f>_xlfn.IFNA(FDS(E$7,"FE_ESTIMATE(EPS,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="F48" s="20">
+      <c r="F48" s="19">
         <f>_xlfn.IFNA(FDS(F$7,"FE_ESTIMATE(EPS,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="G48" s="20">
+      <c r="G48" s="19">
         <f>_xlfn.IFNA(FDS(G$7,"FE_ESTIMATE(EPS,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="H48" s="20">
+      <c r="H48" s="19">
         <f>_xlfn.IFNA(FDS(H$7,"FE_ESTIMATE(EPS,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="I48" s="20">
+      <c r="I48" s="19">
         <f>_xlfn.IFNA(FDS(I$7,"FE_ESTIMATE(EPS,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
@@ -13144,23 +13145,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E64" s="20">
+      <c r="E64" s="19">
         <f>_xlfn.IFNA(FDS(E$7,"FE_ESTIMATE(NETDIV,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="F64" s="20">
+      <c r="F64" s="19">
         <f>_xlfn.IFNA(FDS(F$7,"FE_ESTIMATE(NETDIV,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="G64" s="20">
+      <c r="G64" s="19">
         <f>_xlfn.IFNA(FDS(G$7,"FE_ESTIMATE(NETDIV,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="H64" s="20">
+      <c r="H64" s="19">
         <f>_xlfn.IFNA(FDS(H$7,"FE_ESTIMATE(NETDIV,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="I64" s="20">
+      <c r="I64" s="19">
         <f>_xlfn.IFNA(FDS(I$7,"FE_ESTIMATE(NETDIV,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
@@ -13182,23 +13183,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E65" s="20">
+      <c r="E65" s="19">
         <f>_xlfn.IFNA(FDS(E$7,"FE_ESTIMATE(BPS_TANG,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="F65" s="20">
+      <c r="F65" s="19">
         <f>_xlfn.IFNA(FDS(F$7,"FE_ESTIMATE(BPS_TANG,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="G65" s="20">
+      <c r="G65" s="19">
         <f>_xlfn.IFNA(FDS(G$7,"FE_ESTIMATE(BPS_TANG,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="H65" s="20">
+      <c r="H65" s="19">
         <f>_xlfn.IFNA(FDS(H$7,"FE_ESTIMATE(BPS_TANG,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="I65" s="20">
+      <c r="I65" s="19">
         <f>_xlfn.IFNA(FDS(I$7,"FE_ESTIMATE(BPS_TANG,MEAN,ANN_ROLL,"&amp;$C$4&amp;",NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
@@ -13402,23 +13403,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E72" s="20">
+      <c r="E72" s="19">
         <f>_xlfn.IFNA(FDS(E$7,"FE_ESTIMATE(EPS,MEAN,QTR_ROLL,+1,0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="F72" s="20">
+      <c r="F72" s="19">
         <f>_xlfn.IFNA(FDS(F$7,"FE_ESTIMATE(EPS,MEAN,QTR_ROLL,+1,0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="G72" s="20">
+      <c r="G72" s="19">
         <f>_xlfn.IFNA(FDS(G$7,"FE_ESTIMATE(EPS,MEAN,QTR_ROLL,+1,0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="H72" s="20">
+      <c r="H72" s="19">
         <f>_xlfn.IFNA(FDS(H$7,"FE_ESTIMATE(EPS,MEAN,QTR_ROLL,+1,0,,,'')"),"-")</f>
         <v/>
       </c>
-      <c r="I72" s="20">
+      <c r="I72" s="19">
         <f>_xlfn.IFNA(FDS(I$7,"FE_ESTIMATE(EPS,MEAN,QTR_ROLL,+1,0,,,'')"),"-")</f>
         <v/>
       </c>
@@ -13531,23 +13532,23 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E76" s="20">
+      <c r="E76" s="19">
         <f>_xlfn.IFNA(FDS(E$7,"FE_ESTIMATE(EPS,MEAN,LTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="F76" s="20">
+      <c r="F76" s="19">
         <f>_xlfn.IFNA(FDS(F$7,"FE_ESTIMATE(EPS,MEAN,LTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="G76" s="20">
+      <c r="G76" s="19">
         <f>_xlfn.IFNA(FDS(G$7,"FE_ESTIMATE(EPS,MEAN,LTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="H76" s="20">
+      <c r="H76" s="19">
         <f>_xlfn.IFNA(FDS(H$7,"FE_ESTIMATE(EPS,MEAN,LTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
-      <c r="I76" s="20">
+      <c r="I76" s="19">
         <f>_xlfn.IFNA(FDS(I$7,"FE_ESTIMATE(EPS,MEAN,LTMA,,NOW,,,'CURRENCY=USD')"),"-")</f>
         <v/>
       </c>
@@ -13685,7 +13686,7 @@
           <t>Ticker</t>
         </is>
       </c>
-      <c r="C3" s="23" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>HBAN</t>
         </is>
@@ -14065,21 +14066,21 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E16" s="20">
+      <c r="E16" s="19">
         <f>FDSRC("-",$C$3,"FE_TIMESERIES(EPS,MEAN,"&amp;$E$5&amp;","&amp;$P$5&amp;",FQ,'BKRACTMED=1,WIN=0,CURRENCY=RPT,UNITS=AUTO,DATE=NOW')")</f>
         <v/>
       </c>
-      <c r="F16" s="20" t="n"/>
-      <c r="G16" s="20" t="n"/>
-      <c r="H16" s="20" t="n"/>
-      <c r="I16" s="20" t="n"/>
-      <c r="J16" s="20" t="n"/>
-      <c r="K16" s="20" t="n"/>
-      <c r="L16" s="20" t="n"/>
-      <c r="M16" s="20" t="n"/>
-      <c r="N16" s="20" t="n"/>
-      <c r="O16" s="20" t="n"/>
-      <c r="P16" s="20" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="n"/>
+      <c r="H16" s="19" t="n"/>
+      <c r="I16" s="19" t="n"/>
+      <c r="J16" s="19" t="n"/>
+      <c r="K16" s="19" t="n"/>
+      <c r="L16" s="19" t="n"/>
+      <c r="M16" s="19" t="n"/>
+      <c r="N16" s="19" t="n"/>
+      <c r="O16" s="19" t="n"/>
+      <c r="P16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr"/>
@@ -14098,21 +14099,21 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E17" s="20">
+      <c r="E17" s="19">
         <f>FDSRC("-",$C$3,"FE_TIMESERIES(CUSTOM_EPS,MEAN,"&amp;$E$5&amp;","&amp;$P$5&amp;",FQ,'BKRACTMED=1,WIN=0,CURRENCY=RPT,UNITS=AUTO,DATE=NOW')")</f>
         <v/>
       </c>
-      <c r="F17" s="20" t="n"/>
-      <c r="G17" s="20" t="n"/>
-      <c r="H17" s="20" t="n"/>
-      <c r="I17" s="20" t="n"/>
-      <c r="J17" s="20" t="n"/>
-      <c r="K17" s="20" t="n"/>
-      <c r="L17" s="20" t="n"/>
-      <c r="M17" s="20" t="n"/>
-      <c r="N17" s="20" t="n"/>
-      <c r="O17" s="20" t="n"/>
-      <c r="P17" s="20" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="19" t="n"/>
+      <c r="H17" s="19" t="n"/>
+      <c r="I17" s="19" t="n"/>
+      <c r="J17" s="19" t="n"/>
+      <c r="K17" s="19" t="n"/>
+      <c r="L17" s="19" t="n"/>
+      <c r="M17" s="19" t="n"/>
+      <c r="N17" s="19" t="n"/>
+      <c r="O17" s="19" t="n"/>
+      <c r="P17" s="19" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr"/>
@@ -14681,21 +14682,21 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E36" s="20">
+      <c r="E36" s="19">
         <f>FDSRC("-",$C$3,"FE_TIMESERIES(BPS_TANG,MEAN,"&amp;$E$5&amp;","&amp;$P$5&amp;",FQ,'BKRACTMED=1,WIN=0,CURRENCY=RPT,UNITS=AUTO,DATE=NOW')")</f>
         <v/>
       </c>
-      <c r="F36" s="20" t="n"/>
-      <c r="G36" s="20" t="n"/>
-      <c r="H36" s="20" t="n"/>
-      <c r="I36" s="20" t="n"/>
-      <c r="J36" s="20" t="n"/>
-      <c r="K36" s="20" t="n"/>
-      <c r="L36" s="20" t="n"/>
-      <c r="M36" s="20" t="n"/>
-      <c r="N36" s="20" t="n"/>
-      <c r="O36" s="20" t="n"/>
-      <c r="P36" s="20" t="n"/>
+      <c r="F36" s="19" t="n"/>
+      <c r="G36" s="19" t="n"/>
+      <c r="H36" s="19" t="n"/>
+      <c r="I36" s="19" t="n"/>
+      <c r="J36" s="19" t="n"/>
+      <c r="K36" s="19" t="n"/>
+      <c r="L36" s="19" t="n"/>
+      <c r="M36" s="19" t="n"/>
+      <c r="N36" s="19" t="n"/>
+      <c r="O36" s="19" t="n"/>
+      <c r="P36" s="19" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr"/>
@@ -15044,21 +15045,21 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="E48" s="20">
+      <c r="E48" s="19">
         <f>FDSRC("-",$C$3,"FE_TIMESERIES(NETDIV,MEAN,"&amp;$E$5&amp;","&amp;$P$5&amp;",FQ,'BKRACTMED=1,WIN=0,CURRENCY=RPT,UNITS=AUTO,DATE=NOW')")</f>
         <v/>
       </c>
-      <c r="F48" s="20" t="n"/>
-      <c r="G48" s="20" t="n"/>
-      <c r="H48" s="20" t="n"/>
-      <c r="I48" s="20" t="n"/>
-      <c r="J48" s="20" t="n"/>
-      <c r="K48" s="20" t="n"/>
-      <c r="L48" s="20" t="n"/>
-      <c r="M48" s="20" t="n"/>
-      <c r="N48" s="20" t="n"/>
-      <c r="O48" s="20" t="n"/>
-      <c r="P48" s="20" t="n"/>
+      <c r="F48" s="19" t="n"/>
+      <c r="G48" s="19" t="n"/>
+      <c r="H48" s="19" t="n"/>
+      <c r="I48" s="19" t="n"/>
+      <c r="J48" s="19" t="n"/>
+      <c r="K48" s="19" t="n"/>
+      <c r="L48" s="19" t="n"/>
+      <c r="M48" s="19" t="n"/>
+      <c r="N48" s="19" t="n"/>
+      <c r="O48" s="19" t="n"/>
+      <c r="P48" s="19" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="14" t="inlineStr">
@@ -15094,26 +15095,26 @@
           <t>FE_TIMESERIES_GUIDANCE(COST_INCOME,LOW)</t>
         </is>
       </c>
-      <c r="D50" s="19" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="E50" s="18">
         <f>FDSRC("-",$C$3,"FE_TIMESERIES_GUIDANCE(COST_INCOME,LOW,"&amp;$E$5&amp;","&amp;$P$5&amp;",FQ,'BKRACTMED=1,WIN=0,CURRENCY=RPT,UNITS=AUTO,DATE=NOW')")</f>
         <v/>
       </c>
-      <c r="F50" s="28" t="n"/>
-      <c r="G50" s="28" t="n"/>
-      <c r="H50" s="28" t="n"/>
-      <c r="I50" s="28" t="n"/>
-      <c r="J50" s="28" t="n"/>
-      <c r="K50" s="28" t="n"/>
-      <c r="L50" s="28" t="n"/>
-      <c r="M50" s="28" t="n"/>
-      <c r="N50" s="28" t="n"/>
-      <c r="O50" s="28" t="n"/>
-      <c r="P50" s="28" t="n"/>
+      <c r="F50" s="27" t="n"/>
+      <c r="G50" s="27" t="n"/>
+      <c r="H50" s="27" t="n"/>
+      <c r="I50" s="27" t="n"/>
+      <c r="J50" s="27" t="n"/>
+      <c r="K50" s="27" t="n"/>
+      <c r="L50" s="27" t="n"/>
+      <c r="M50" s="27" t="n"/>
+      <c r="N50" s="27" t="n"/>
+      <c r="O50" s="27" t="n"/>
+      <c r="P50" s="27" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E7:P50">

</xml_diff>